<commit_message>
Finished PCB and starting CAD
</commit_message>
<xml_diff>
--- a/PhantomBOM.xlsx
+++ b/PhantomBOM.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7bd69513486a8436/Documents/Phantom/Phantom/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="84" documentId="8_{C253D126-2466-4473-A8D9-932367B4E877}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BB534472-573D-40F1-AF9C-C8B0C4811D4B}"/>
+  <xr:revisionPtr revIDLastSave="135" documentId="8_{C253D126-2466-4473-A8D9-932367B4E877}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1E9820A6-E2B7-485A-8FDD-BB43185EF14A}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="732" yWindow="732" windowWidth="17280" windowHeight="9960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="75">
   <si>
     <t>Item Name</t>
   </si>
@@ -100,12 +100,6 @@
     <t>TH1</t>
   </si>
   <si>
-    <t>MCR-B-S-RA-SMT-EH4B-T/R</t>
-  </si>
-  <si>
-    <t>https://www.digikey.com/en/products/detail/adam-tech/MCR-B-S-RA-SMT-EH4B-T-R/9832095</t>
-  </si>
-  <si>
     <t>USB</t>
   </si>
   <si>
@@ -185,6 +179,72 @@
   </si>
   <si>
     <t>Coin battery holder</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/sparkfun-electronics/15141/10130910</t>
+  </si>
+  <si>
+    <t>Rotary Encoder</t>
+  </si>
+  <si>
+    <t>SW3</t>
+  </si>
+  <si>
+    <t>L101011MS02Q</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/c-k/L101011MS02Q/484142</t>
+  </si>
+  <si>
+    <t>Power Switch</t>
+  </si>
+  <si>
+    <t>SW4</t>
+  </si>
+  <si>
+    <t>DX4R005HJ5R2000</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/jae-electronics/DX4R005HJ5R2000/3903227</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/hirose-electric-co-ltd/FH33-10S-0-5SH-10/1305324</t>
+  </si>
+  <si>
+    <t>Screen Connector</t>
+  </si>
+  <si>
+    <t>FH33-10S-0.5SH(10)</t>
+  </si>
+  <si>
+    <t>AGGP.25F.07.0060A</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/taoglas-limited/aggp-25f-07-0060a/3083243</t>
+  </si>
+  <si>
+    <t>GPS Antenna</t>
+  </si>
+  <si>
+    <t>U.FL-R-SMT-K(895)</t>
+  </si>
+  <si>
+    <t>GPS Antenna Connector</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/products/detail/hirose-electric-co-ltd/U-FL-R-SMT-1-10/2391570</t>
+  </si>
+  <si>
+    <t>https://www.digikey.com/en/models/926641?tab=snapmagic</t>
+  </si>
+  <si>
+    <t>Battery Connector</t>
+  </si>
+  <si>
+    <t>J3</t>
+  </si>
+  <si>
+    <t>B2B-PH-SM4-TB</t>
   </si>
 </sst>
 </file>
@@ -592,22 +652,22 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>26</v>
+        <v>60</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
       <c r="C5" s="2">
-        <v>0.65</v>
+        <v>0.8</v>
       </c>
       <c r="D5" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="E5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" t="s">
         <v>27</v>
-      </c>
-      <c r="E5" t="s">
-        <v>28</v>
-      </c>
-      <c r="F5" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -624,7 +684,7 @@
         <v>12</v>
       </c>
       <c r="E6" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="F6" t="s">
         <v>24</v>
@@ -652,7 +712,7 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B8">
         <v>1</v>
@@ -661,18 +721,18 @@
         <v>0.44</v>
       </c>
       <c r="D8" t="s">
+        <v>28</v>
+      </c>
+      <c r="E8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F8" t="s">
         <v>30</v>
-      </c>
-      <c r="E8" t="s">
-        <v>31</v>
-      </c>
-      <c r="F8" t="s">
-        <v>32</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B9" s="1">
         <v>1</v>
@@ -681,18 +741,18 @@
         <v>1.05</v>
       </c>
       <c r="D9" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="F9" s="1" t="s">
         <v>35</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B10">
         <v>1</v>
@@ -700,19 +760,19 @@
       <c r="C10" s="2">
         <v>2.41</v>
       </c>
-      <c r="D10" t="s">
-        <v>38</v>
+      <c r="D10" s="7" t="s">
+        <v>36</v>
       </c>
       <c r="E10" t="s">
+        <v>37</v>
+      </c>
+      <c r="F10" t="s">
         <v>39</v>
-      </c>
-      <c r="F10" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B11">
         <v>2</v>
@@ -721,18 +781,18 @@
         <v>1.17</v>
       </c>
       <c r="D11" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E11" t="s">
+        <v>43</v>
+      </c>
+      <c r="F11" t="s">
         <v>44</v>
-      </c>
-      <c r="E11" t="s">
-        <v>45</v>
-      </c>
-      <c r="F11" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B12">
         <v>1</v>
@@ -740,19 +800,19 @@
       <c r="C12" s="2">
         <v>1.27</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="E12" t="s">
+        <v>47</v>
+      </c>
+      <c r="F12" t="s">
         <v>48</v>
-      </c>
-      <c r="E12" t="s">
-        <v>49</v>
-      </c>
-      <c r="F12" t="s">
-        <v>50</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B13">
         <v>1</v>
@@ -760,33 +820,132 @@
       <c r="C13" s="2">
         <v>1.37</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="E13" t="s">
         <v>52</v>
       </c>
-      <c r="E13" t="s">
+      <c r="F13" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14">
+        <v>15141</v>
+      </c>
+      <c r="B14">
+        <v>1</v>
+      </c>
+      <c r="C14" s="2">
+        <v>4.96</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="E14" t="s">
         <v>54</v>
       </c>
-      <c r="F13" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C14" s="2"/>
+      <c r="F14" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C15" s="2"/>
+      <c r="A15" t="s">
+        <v>56</v>
+      </c>
+      <c r="B15">
+        <v>1</v>
+      </c>
+      <c r="C15" s="2">
+        <v>3.97</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="E15" t="s">
+        <v>58</v>
+      </c>
+      <c r="F15" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C16" s="2"/>
+      <c r="A16" t="s">
+        <v>64</v>
+      </c>
+      <c r="B16">
+        <v>1</v>
+      </c>
+      <c r="C16" s="2">
+        <v>1.22</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="E16" t="s">
+        <v>63</v>
+      </c>
+      <c r="F16" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C17" s="2"/>
+      <c r="A17" t="s">
+        <v>65</v>
+      </c>
+      <c r="B17">
+        <v>1</v>
+      </c>
+      <c r="C17" s="2">
+        <v>19.3</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="E17" t="s">
+        <v>67</v>
+      </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C18" s="2"/>
+      <c r="A18" t="s">
+        <v>68</v>
+      </c>
+      <c r="B18">
+        <v>1</v>
+      </c>
+      <c r="C18" s="2">
+        <v>1.29</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="E18" t="s">
+        <v>69</v>
+      </c>
+      <c r="F18" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="C19" s="2"/>
+      <c r="A19" t="s">
+        <v>74</v>
+      </c>
+      <c r="B19">
+        <v>1</v>
+      </c>
+      <c r="C19" s="2">
+        <v>0.47</v>
+      </c>
+      <c r="D19" t="s">
+        <v>71</v>
+      </c>
+      <c r="E19" t="s">
+        <v>72</v>
+      </c>
+      <c r="F19" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="C20" s="2"/>
@@ -3749,6 +3908,15 @@
     <hyperlink ref="D7" r:id="rId5" xr:uid="{C3C00219-F6A4-49A2-ACE4-A106BF51F8FC}"/>
     <hyperlink ref="D9" r:id="rId6" xr:uid="{BB613A42-BF29-46C8-907A-BEAAC1535931}"/>
     <hyperlink ref="D11" r:id="rId7" display="https://www.digikey.com/en/products/detail/omron-electronics-inc-emc-div/B3U-1100P/1534339?gclsrc=aw.ds&amp;gad_source=1&amp;gad_campaignid=20234014242&amp;gbraid=0AAAAADrbLlis3Cz40t9hjOioxPaFcy7Si&amp;gclid=Cj0KCQjw9ZLSBhCcARIsAEhGKgMMIXBGDglw2WMnyUzLqVsnmpcDYfhjn9ClIkeviY8wOCGYYd3g9hoaAp_GEALw_wcB" xr:uid="{11DBBCC3-C1AB-458D-A13D-AB15568895F1}"/>
+    <hyperlink ref="D14" r:id="rId8" xr:uid="{6A6E6808-941F-4C31-B55C-25EEA0A532B9}"/>
+    <hyperlink ref="D15" r:id="rId9" xr:uid="{A7614A74-8585-4583-88C7-7C64D434FE6B}"/>
+    <hyperlink ref="D12" r:id="rId10" xr:uid="{0DA95EDA-91D1-42C6-97C8-6FB121587AFD}"/>
+    <hyperlink ref="D5" r:id="rId11" xr:uid="{BA27FBC6-665B-44D1-9D26-90D79BF0713C}"/>
+    <hyperlink ref="D18" r:id="rId12" xr:uid="{D5895E37-1669-4BE0-9DCE-10CD65FA4419}"/>
+    <hyperlink ref="D16" r:id="rId13" xr:uid="{F205D0CD-AB7B-445E-B35A-43F47E1629F6}"/>
+    <hyperlink ref="D13" r:id="rId14" xr:uid="{A0292413-CD35-4D7B-A741-27405701ED7D}"/>
+    <hyperlink ref="D10" r:id="rId15" xr:uid="{2E1AE9FB-8DAC-43A4-998B-E8A7954B5508}"/>
+    <hyperlink ref="D17" r:id="rId16" xr:uid="{976EA0AD-2FAA-4CD8-979D-2E724CFC378C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>